<commit_message>
upload: seniority for 2025-11-05 (051125/Crew_Pairing.xlsx)
</commit_message>
<xml_diff>
--- a/outputs/2025-11-05/inputs/seniority.xlsx
+++ b/outputs/2025-11-05/inputs/seniority.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Crew Sched and BD Shared Folder\2025\November\Processed data\051125\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Flight Operations\Crew Sched and BD Shared Folder\2025\November\Input Files\KTree\051125\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1254E91-39CD-47FC-89DA-300F6002B3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{155A15CD-8224-41CC-9A9E-3949BD606080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03228E58-5772-4D09-93C2-473CFEDC8A2C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{03228E58-5772-4D09-93C2-473CFEDC8A2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -1458,7 +1455,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1982,12 +1979,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1E1265A-02B7-4E01-9694-14673A775217}">
   <dimension ref="A1:C464"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1998,7 +1995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -2009,7 +2006,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -2020,7 +2017,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -2031,7 +2028,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -2042,7 +2039,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -2053,7 +2050,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
@@ -2064,7 +2061,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
@@ -2075,7 +2072,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
@@ -2086,7 +2083,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
@@ -2097,7 +2094,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>12</v>
       </c>
@@ -2108,7 +2105,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
@@ -2119,7 +2116,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>14</v>
       </c>
@@ -2130,7 +2127,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
@@ -2141,7 +2138,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
@@ -2152,7 +2149,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>17</v>
       </c>
@@ -2163,7 +2160,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>18</v>
       </c>
@@ -2174,7 +2171,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>19</v>
       </c>
@@ -2185,7 +2182,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
@@ -2196,7 +2193,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>21</v>
       </c>
@@ -2207,7 +2204,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>22</v>
       </c>
@@ -2218,7 +2215,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>23</v>
       </c>
@@ -2229,7 +2226,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>24</v>
       </c>
@@ -2240,7 +2237,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>25</v>
       </c>
@@ -2251,7 +2248,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>
@@ -2262,7 +2259,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>27</v>
       </c>
@@ -2273,7 +2270,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>28</v>
       </c>
@@ -2284,7 +2281,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>29</v>
       </c>
@@ -2295,7 +2292,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>30</v>
       </c>
@@ -2306,7 +2303,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>31</v>
       </c>
@@ -2317,7 +2314,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>32</v>
       </c>
@@ -2328,7 +2325,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>33</v>
       </c>
@@ -2339,7 +2336,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>34</v>
       </c>
@@ -2350,7 +2347,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>35</v>
       </c>
@@ -2361,7 +2358,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>36</v>
       </c>
@@ -2372,7 +2369,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>37</v>
       </c>
@@ -2383,7 +2380,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>38</v>
       </c>
@@ -2394,7 +2391,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>39</v>
       </c>
@@ -2405,7 +2402,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>40</v>
       </c>
@@ -2416,7 +2413,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>41</v>
       </c>
@@ -2427,7 +2424,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>42</v>
       </c>
@@ -2438,7 +2435,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>43</v>
       </c>
@@ -2449,7 +2446,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>44</v>
       </c>
@@ -2460,7 +2457,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>45</v>
       </c>
@@ -2471,7 +2468,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>46</v>
       </c>
@@ -2482,7 +2479,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>47</v>
       </c>
@@ -2493,7 +2490,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>48</v>
       </c>
@@ -2504,7 +2501,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>49</v>
       </c>
@@ -2515,7 +2512,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>50</v>
       </c>
@@ -2526,7 +2523,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>51</v>
       </c>
@@ -2537,7 +2534,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>52</v>
       </c>
@@ -2548,7 +2545,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>53</v>
       </c>
@@ -2559,7 +2556,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>54</v>
       </c>
@@ -2570,7 +2567,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>55</v>
       </c>
@@ -2581,7 +2578,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>56</v>
       </c>
@@ -2592,7 +2589,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>57</v>
       </c>
@@ -2603,7 +2600,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>58</v>
       </c>
@@ -2614,7 +2611,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>59</v>
       </c>
@@ -2625,7 +2622,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>60</v>
       </c>
@@ -2636,7 +2633,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>61</v>
       </c>
@@ -2647,7 +2644,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>62</v>
       </c>
@@ -2658,7 +2655,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>63</v>
       </c>
@@ -2669,7 +2666,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>64</v>
       </c>
@@ -2680,7 +2677,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>65</v>
       </c>
@@ -2691,7 +2688,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>66</v>
       </c>
@@ -2702,7 +2699,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>67</v>
       </c>
@@ -2713,7 +2710,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>68</v>
       </c>
@@ -2724,7 +2721,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>69</v>
       </c>
@@ -2735,7 +2732,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>70</v>
       </c>
@@ -2746,7 +2743,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>71</v>
       </c>
@@ -2757,7 +2754,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>72</v>
       </c>
@@ -2768,7 +2765,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>73</v>
       </c>
@@ -2779,7 +2776,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>74</v>
       </c>
@@ -2790,7 +2787,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>75</v>
       </c>
@@ -2801,7 +2798,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>76</v>
       </c>
@@ -2812,7 +2809,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>77</v>
       </c>
@@ -2823,7 +2820,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>78</v>
       </c>
@@ -2834,7 +2831,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>79</v>
       </c>
@@ -2845,7 +2842,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>80</v>
       </c>
@@ -2856,7 +2853,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>81</v>
       </c>
@@ -2867,7 +2864,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>82</v>
       </c>
@@ -2878,7 +2875,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>83</v>
       </c>
@@ -2889,7 +2886,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>84</v>
       </c>
@@ -2900,7 +2897,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>85</v>
       </c>
@@ -2911,7 +2908,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
         <v>86</v>
       </c>
@@ -2922,7 +2919,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>87</v>
       </c>
@@ -2933,7 +2930,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>88</v>
       </c>
@@ -2944,7 +2941,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>89</v>
       </c>
@@ -2955,7 +2952,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>90</v>
       </c>
@@ -2966,7 +2963,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>91</v>
       </c>
@@ -2977,7 +2974,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>92</v>
       </c>
@@ -2988,7 +2985,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>93</v>
       </c>
@@ -2999,7 +2996,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>94</v>
       </c>
@@ -3010,7 +3007,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>95</v>
       </c>
@@ -3021,7 +3018,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>96</v>
       </c>
@@ -3032,7 +3029,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>97</v>
       </c>
@@ -3043,7 +3040,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>98</v>
       </c>
@@ -3054,7 +3051,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>99</v>
       </c>
@@ -3065,7 +3062,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
         <v>100</v>
       </c>
@@ -3076,7 +3073,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>101</v>
       </c>
@@ -3087,7 +3084,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
         <v>102</v>
       </c>
@@ -3098,7 +3095,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>103</v>
       </c>
@@ -3109,7 +3106,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>104</v>
       </c>
@@ -3120,7 +3117,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
         <v>105</v>
       </c>
@@ -3131,7 +3128,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>106</v>
       </c>
@@ -3142,7 +3139,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
         <v>107</v>
       </c>
@@ -3153,7 +3150,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" s="4" t="s">
         <v>108</v>
       </c>
@@ -3164,7 +3161,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>109</v>
       </c>
@@ -3175,7 +3172,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
         <v>110</v>
       </c>
@@ -3186,7 +3183,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
         <v>111</v>
       </c>
@@ -3197,7 +3194,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
         <v>112</v>
       </c>
@@ -3208,7 +3205,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
         <v>113</v>
       </c>
@@ -3219,7 +3216,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>114</v>
       </c>
@@ -3230,7 +3227,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
         <v>115</v>
       </c>
@@ -3241,7 +3238,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
         <v>116</v>
       </c>
@@ -3252,7 +3249,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
         <v>117</v>
       </c>
@@ -3263,7 +3260,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
         <v>118</v>
       </c>
@@ -3274,7 +3271,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>119</v>
       </c>
@@ -3285,7 +3282,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>120</v>
       </c>
@@ -3296,7 +3293,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
         <v>162</v>
       </c>
@@ -3307,7 +3304,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" s="4" t="s">
         <v>163</v>
       </c>
@@ -3318,7 +3315,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>164</v>
       </c>
@@ -3329,7 +3326,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" s="4" t="s">
         <v>165</v>
       </c>
@@ -3340,7 +3337,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
         <v>166</v>
       </c>
@@ -3351,7 +3348,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
         <v>167</v>
       </c>
@@ -3362,7 +3359,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" s="4" t="s">
         <v>168</v>
       </c>
@@ -3373,7 +3370,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" s="4" t="s">
         <v>169</v>
       </c>
@@ -3384,7 +3381,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="128" spans="1:3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" s="10" t="s">
         <v>170</v>
       </c>
@@ -3395,7 +3392,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="129" spans="1:3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" s="4" t="s">
         <v>171</v>
       </c>
@@ -3406,7 +3403,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="130" spans="1:3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" s="4" t="s">
         <v>172</v>
       </c>
@@ -3417,7 +3414,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="131" spans="1:3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
         <v>173</v>
       </c>
@@ -3428,7 +3425,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="132" spans="1:3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" s="4" t="s">
         <v>174</v>
       </c>
@@ -3439,7 +3436,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="133" spans="1:3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" s="4" t="s">
         <v>175</v>
       </c>
@@ -3450,7 +3447,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="134" spans="1:3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" s="10" t="s">
         <v>176</v>
       </c>
@@ -3461,7 +3458,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" s="4" t="s">
         <v>177</v>
       </c>
@@ -3472,7 +3469,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="136" spans="1:3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" s="4" t="s">
         <v>178</v>
       </c>
@@ -3483,7 +3480,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="137" spans="1:3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
         <v>179</v>
       </c>
@@ -3494,7 +3491,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
         <v>180</v>
       </c>
@@ -3505,7 +3502,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" s="4" t="s">
         <v>181</v>
       </c>
@@ -3516,7 +3513,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" s="5" t="s">
         <v>182</v>
       </c>
@@ -3527,7 +3524,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
         <v>183</v>
       </c>
@@ -3538,7 +3535,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
         <v>184</v>
       </c>
@@ -3549,7 +3546,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
         <v>185</v>
       </c>
@@ -3560,7 +3557,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" s="4" t="s">
         <v>186</v>
       </c>
@@ -3571,7 +3568,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="145" spans="1:3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" s="5" t="s">
         <v>187</v>
       </c>
@@ -3582,7 +3579,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="146" spans="1:3">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" s="4" t="s">
         <v>188</v>
       </c>
@@ -3593,7 +3590,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="147" spans="1:3">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" s="5" t="s">
         <v>189</v>
       </c>
@@ -3604,7 +3601,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="148" spans="1:3">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" s="5" t="s">
         <v>190</v>
       </c>
@@ -3615,7 +3612,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="149" spans="1:3">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" s="5" t="s">
         <v>191</v>
       </c>
@@ -3626,7 +3623,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="150" spans="1:3">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" s="5" t="s">
         <v>192</v>
       </c>
@@ -3637,7 +3634,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="151" spans="1:3">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" s="5" t="s">
         <v>193</v>
       </c>
@@ -3648,7 +3645,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="152" spans="1:3">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" s="5" t="s">
         <v>194</v>
       </c>
@@ -3659,7 +3656,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="153" spans="1:3">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" s="5" t="s">
         <v>195</v>
       </c>
@@ -3670,7 +3667,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="154" spans="1:3">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
         <v>196</v>
       </c>
@@ -3681,7 +3678,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="155" spans="1:3">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
         <v>197</v>
       </c>
@@ -3692,7 +3689,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="156" spans="1:3">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
         <v>198</v>
       </c>
@@ -3703,7 +3700,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="157" spans="1:3">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" s="4" t="s">
         <v>199</v>
       </c>
@@ -3714,7 +3711,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="158" spans="1:3">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
         <v>200</v>
       </c>
@@ -3725,7 +3722,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="159" spans="1:3">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" s="4" t="s">
         <v>201</v>
       </c>
@@ -3736,7 +3733,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="160" spans="1:3">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" s="4" t="s">
         <v>202</v>
       </c>
@@ -3747,7 +3744,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="161" spans="1:3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
         <v>203</v>
       </c>
@@ -3758,7 +3755,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="162" spans="1:3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
         <v>204</v>
       </c>
@@ -3769,7 +3766,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="163" spans="1:3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
         <v>205</v>
       </c>
@@ -3780,7 +3777,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="164" spans="1:3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" s="10" t="s">
         <v>206</v>
       </c>
@@ -3791,7 +3788,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" s="4" t="s">
         <v>207</v>
       </c>
@@ -3802,7 +3799,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" s="4" t="s">
         <v>208</v>
       </c>
@@ -3813,7 +3810,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" s="4" t="s">
         <v>209</v>
       </c>
@@ -3824,7 +3821,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="168" spans="1:3">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" s="4" t="s">
         <v>210</v>
       </c>
@@ -3835,7 +3832,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" s="4" t="s">
         <v>211</v>
       </c>
@@ -3846,7 +3843,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="170" spans="1:3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" s="4" t="s">
         <v>212</v>
       </c>
@@ -3857,7 +3854,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" s="4" t="s">
         <v>213</v>
       </c>
@@ -3868,7 +3865,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" s="4" t="s">
         <v>214</v>
       </c>
@@ -3879,7 +3876,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="173" spans="1:3">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" s="4" t="s">
         <v>215</v>
       </c>
@@ -3890,7 +3887,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="174" spans="1:3">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" s="4" t="s">
         <v>216</v>
       </c>
@@ -3901,7 +3898,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" s="4" t="s">
         <v>217</v>
       </c>
@@ -3912,7 +3909,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="176" spans="1:3">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" s="4" t="s">
         <v>218</v>
       </c>
@@ -3923,7 +3920,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" s="4" t="s">
         <v>219</v>
       </c>
@@ -3934,7 +3931,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" s="4" t="s">
         <v>220</v>
       </c>
@@ -3945,7 +3942,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" s="4" t="s">
         <v>221</v>
       </c>
@@ -3956,7 +3953,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" s="10" t="s">
         <v>222</v>
       </c>
@@ -3967,7 +3964,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" s="4" t="s">
         <v>223</v>
       </c>
@@ -3978,7 +3975,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="182" spans="1:3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" s="10" t="s">
         <v>224</v>
       </c>
@@ -3989,7 +3986,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" s="4" t="s">
         <v>225</v>
       </c>
@@ -4000,7 +3997,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" s="4" t="s">
         <v>226</v>
       </c>
@@ -4011,7 +4008,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" s="4" t="s">
         <v>227</v>
       </c>
@@ -4022,7 +4019,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="186" spans="1:3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" s="4" t="s">
         <v>228</v>
       </c>
@@ -4033,7 +4030,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" s="4" t="s">
         <v>229</v>
       </c>
@@ -4044,7 +4041,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" s="4" t="s">
         <v>230</v>
       </c>
@@ -4055,7 +4052,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="189" spans="1:3">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" s="4" t="s">
         <v>231</v>
       </c>
@@ -4066,7 +4063,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" s="4" t="s">
         <v>232</v>
       </c>
@@ -4077,7 +4074,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" s="4" t="s">
         <v>233</v>
       </c>
@@ -4088,7 +4085,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="192" spans="1:3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" s="4" t="s">
         <v>234</v>
       </c>
@@ -4099,7 +4096,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" s="4" t="s">
         <v>235</v>
       </c>
@@ -4110,7 +4107,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" s="4" t="s">
         <v>236</v>
       </c>
@@ -4121,7 +4118,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" s="4" t="s">
         <v>237</v>
       </c>
@@ -4132,7 +4129,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="196" spans="1:3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" s="4" t="s">
         <v>238</v>
       </c>
@@ -4143,7 +4140,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" s="10" t="s">
         <v>239</v>
       </c>
@@ -4154,7 +4151,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="198" spans="1:3">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" s="4" t="s">
         <v>240</v>
       </c>
@@ -4165,7 +4162,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="199" spans="1:3">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" s="4" t="s">
         <v>241</v>
       </c>
@@ -4176,7 +4173,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="200" spans="1:3">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" s="4" t="s">
         <v>242</v>
       </c>
@@ -4187,7 +4184,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="201" spans="1:3">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" s="4" t="s">
         <v>243</v>
       </c>
@@ -4198,7 +4195,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="202" spans="1:3">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" s="4" t="s">
         <v>244</v>
       </c>
@@ -4209,7 +4206,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="203" spans="1:3">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" s="4" t="s">
         <v>245</v>
       </c>
@@ -4220,7 +4217,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="204" spans="1:3">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" s="4" t="s">
         <v>246</v>
       </c>
@@ -4231,7 +4228,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="205" spans="1:3">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205" s="4" t="s">
         <v>247</v>
       </c>
@@ -4242,7 +4239,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="206" spans="1:3">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" s="4" t="s">
         <v>248</v>
       </c>
@@ -4253,7 +4250,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="207" spans="1:3">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" s="4" t="s">
         <v>249</v>
       </c>
@@ -4264,7 +4261,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="208" spans="1:3">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" s="4" t="s">
         <v>250</v>
       </c>
@@ -4275,7 +4272,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="209" spans="1:3">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209" s="4" t="s">
         <v>251</v>
       </c>
@@ -4286,7 +4283,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="210" spans="1:3">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A210" s="4" t="s">
         <v>252</v>
       </c>
@@ -4297,7 +4294,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="211" spans="1:3">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211" s="4" t="s">
         <v>253</v>
       </c>
@@ -4308,7 +4305,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="212" spans="1:3">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212" s="4" t="s">
         <v>254</v>
       </c>
@@ -4319,7 +4316,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="213" spans="1:3">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213" s="4" t="s">
         <v>255</v>
       </c>
@@ -4330,7 +4327,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="214" spans="1:3">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214" s="4" t="s">
         <v>256</v>
       </c>
@@ -4341,7 +4338,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="215" spans="1:3">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215" s="4" t="s">
         <v>257</v>
       </c>
@@ -4352,7 +4349,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="216" spans="1:3">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216" s="4" t="s">
         <v>267</v>
       </c>
@@ -4363,7 +4360,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="217" spans="1:3">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217" s="4" t="s">
         <v>312</v>
       </c>
@@ -4374,7 +4371,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="218" spans="1:3">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218" s="4" t="s">
         <v>313</v>
       </c>
@@ -4385,7 +4382,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="219" spans="1:3">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A219" s="4" t="s">
         <v>314</v>
       </c>
@@ -4396,7 +4393,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="220" spans="1:3">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A220" s="4" t="s">
         <v>315</v>
       </c>
@@ -4407,7 +4404,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="221" spans="1:3">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A221" s="4" t="s">
         <v>316</v>
       </c>
@@ -4418,7 +4415,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="222" spans="1:3">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A222" s="4" t="s">
         <v>317</v>
       </c>
@@ -4429,7 +4426,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="223" spans="1:3">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" s="4" t="s">
         <v>318</v>
       </c>
@@ -4440,7 +4437,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="224" spans="1:3">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224" s="4" t="s">
         <v>319</v>
       </c>
@@ -4451,7 +4448,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="225" spans="1:3">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A225" s="4" t="s">
         <v>320</v>
       </c>
@@ -4462,7 +4459,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="226" spans="1:3">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A226" s="4" t="s">
         <v>321</v>
       </c>
@@ -4473,7 +4470,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="227" spans="1:3">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A227" s="4" t="s">
         <v>322</v>
       </c>
@@ -4484,7 +4481,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="228" spans="1:3">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A228" s="4" t="s">
         <v>323</v>
       </c>
@@ -4495,7 +4492,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="229" spans="1:3">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A229" s="4" t="s">
         <v>324</v>
       </c>
@@ -4506,7 +4503,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="230" spans="1:3">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A230" s="4" t="s">
         <v>325</v>
       </c>
@@ -4517,7 +4514,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="231" spans="1:3">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A231" s="4" t="s">
         <v>326</v>
       </c>
@@ -4528,7 +4525,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="232" spans="1:3">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A232" s="4" t="s">
         <v>327</v>
       </c>
@@ -4539,7 +4536,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="233" spans="1:3">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A233" s="4" t="s">
         <v>328</v>
       </c>
@@ -4550,7 +4547,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="234" spans="1:3">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A234" s="4" t="s">
         <v>329</v>
       </c>
@@ -4561,7 +4558,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="235" spans="1:3">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A235" s="4" t="s">
         <v>330</v>
       </c>
@@ -4572,7 +4569,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="236" spans="1:3">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A236" s="4" t="s">
         <v>331</v>
       </c>
@@ -4583,7 +4580,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="237" spans="1:3">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A237" s="4" t="s">
         <v>332</v>
       </c>
@@ -4594,7 +4591,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="238" spans="1:3">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A238" s="4" t="s">
         <v>333</v>
       </c>
@@ -4605,7 +4602,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="239" spans="1:3">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A239" s="4" t="s">
         <v>334</v>
       </c>
@@ -4616,7 +4613,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="240" spans="1:3">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A240" s="4" t="s">
         <v>335</v>
       </c>
@@ -4627,7 +4624,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="241" spans="1:3">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A241" s="4" t="s">
         <v>336</v>
       </c>
@@ -4638,7 +4635,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="242" spans="1:3">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A242" s="4" t="s">
         <v>337</v>
       </c>
@@ -4649,7 +4646,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="243" spans="1:3">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A243" s="4" t="s">
         <v>338</v>
       </c>
@@ -4660,7 +4657,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A244" s="4" t="s">
         <v>339</v>
       </c>
@@ -4671,7 +4668,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="245" spans="1:3">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A245" s="4" t="s">
         <v>340</v>
       </c>
@@ -4682,7 +4679,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="246" spans="1:3">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A246" s="4" t="s">
         <v>341</v>
       </c>
@@ -4693,7 +4690,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="247" spans="1:3">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A247" s="4" t="s">
         <v>342</v>
       </c>
@@ -4704,7 +4701,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="248" spans="1:3">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A248" s="4" t="s">
         <v>343</v>
       </c>
@@ -4715,7 +4712,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="249" spans="1:3">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A249" s="4" t="s">
         <v>344</v>
       </c>
@@ -4726,7 +4723,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="250" spans="1:3">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A250" s="4" t="s">
         <v>345</v>
       </c>
@@ -4737,7 +4734,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="251" spans="1:3">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A251" s="4" t="s">
         <v>346</v>
       </c>
@@ -4748,7 +4745,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="252" spans="1:3">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A252" s="4" t="s">
         <v>347</v>
       </c>
@@ -4759,7 +4756,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="253" spans="1:3">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A253" s="4" t="s">
         <v>348</v>
       </c>
@@ -4770,7 +4767,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="254" spans="1:3">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A254" s="4" t="s">
         <v>349</v>
       </c>
@@ -4781,7 +4778,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="255" spans="1:3">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A255" s="10" t="s">
         <v>350</v>
       </c>
@@ -4792,7 +4789,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="256" spans="1:3">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A256" s="4" t="s">
         <v>351</v>
       </c>
@@ -4803,7 +4800,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="257" spans="1:3">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A257" s="4" t="s">
         <v>352</v>
       </c>
@@ -4814,7 +4811,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="258" spans="1:3">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A258" s="10" t="s">
         <v>353</v>
       </c>
@@ -4825,7 +4822,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="259" spans="1:3">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A259" s="4" t="s">
         <v>354</v>
       </c>
@@ -4836,7 +4833,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="260" spans="1:3">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A260" s="4" t="s">
         <v>355</v>
       </c>
@@ -4847,7 +4844,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="261" spans="1:3">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A261" s="4" t="s">
         <v>356</v>
       </c>
@@ -4858,7 +4855,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="262" spans="1:3">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A262" s="4" t="s">
         <v>357</v>
       </c>
@@ -4869,7 +4866,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="263" spans="1:3">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A263" s="4" t="s">
         <v>358</v>
       </c>
@@ -4880,7 +4877,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="264" spans="1:3">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A264" s="10" t="s">
         <v>359</v>
       </c>
@@ -4891,7 +4888,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="265" spans="1:3">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A265" s="4" t="s">
         <v>360</v>
       </c>
@@ -4902,7 +4899,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="266" spans="1:3">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A266" s="4" t="s">
         <v>361</v>
       </c>
@@ -4913,7 +4910,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="267" spans="1:3">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A267" s="4" t="s">
         <v>362</v>
       </c>
@@ -4924,7 +4921,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="268" spans="1:3">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A268" s="4" t="s">
         <v>363</v>
       </c>
@@ -4935,7 +4932,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="269" spans="1:3">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A269" s="4" t="s">
         <v>364</v>
       </c>
@@ -4946,7 +4943,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="270" spans="1:3">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A270" s="4" t="s">
         <v>365</v>
       </c>
@@ -4957,7 +4954,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="271" spans="1:3">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A271" s="4" t="s">
         <v>366</v>
       </c>
@@ -4968,7 +4965,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="272" spans="1:3">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A272" s="4" t="s">
         <v>367</v>
       </c>
@@ -4979,7 +4976,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="273" spans="1:3">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A273" s="4" t="s">
         <v>368</v>
       </c>
@@ -4990,7 +4987,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="274" spans="1:3">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A274" s="4" t="s">
         <v>369</v>
       </c>
@@ -5001,7 +4998,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="275" spans="1:3">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A275" s="4" t="s">
         <v>370</v>
       </c>
@@ -5012,7 +5009,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="276" spans="1:3">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A276" s="4" t="s">
         <v>371</v>
       </c>
@@ -5023,7 +5020,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="277" spans="1:3">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A277" s="4" t="s">
         <v>372</v>
       </c>
@@ -5034,7 +5031,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A278" s="4" t="s">
         <v>373</v>
       </c>
@@ -5045,7 +5042,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="279" spans="1:3">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A279" s="4" t="s">
         <v>374</v>
       </c>
@@ -5056,7 +5053,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="280" spans="1:3">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A280" s="4" t="s">
         <v>375</v>
       </c>
@@ -5067,7 +5064,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="281" spans="1:3">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A281" s="4" t="s">
         <v>376</v>
       </c>
@@ -5078,7 +5075,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A282" s="4" t="s">
         <v>377</v>
       </c>
@@ -5089,7 +5086,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="283" spans="1:3">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A283" s="4" t="s">
         <v>378</v>
       </c>
@@ -5100,7 +5097,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="284" spans="1:3">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A284" s="4" t="s">
         <v>379</v>
       </c>
@@ -5111,7 +5108,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="285" spans="1:3">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A285" s="4" t="s">
         <v>380</v>
       </c>
@@ -5122,7 +5119,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="286" spans="1:3">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A286" s="4" t="s">
         <v>381</v>
       </c>
@@ -5133,7 +5130,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="287" spans="1:3">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A287" s="4" t="s">
         <v>382</v>
       </c>
@@ -5144,7 +5141,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="288" spans="1:3">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A288" s="4" t="s">
         <v>383</v>
       </c>
@@ -5155,7 +5152,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="289" spans="1:3">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A289" s="4" t="s">
         <v>384</v>
       </c>
@@ -5166,7 +5163,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="290" spans="1:3">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A290" s="4" t="s">
         <v>385</v>
       </c>
@@ -5177,7 +5174,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="291" spans="1:3">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A291" s="4" t="s">
         <v>386</v>
       </c>
@@ -5188,7 +5185,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="292" spans="1:3">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A292" s="4" t="s">
         <v>387</v>
       </c>
@@ -5199,7 +5196,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A293" s="4" t="s">
         <v>388</v>
       </c>
@@ -5210,7 +5207,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="294" spans="1:3">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A294" s="4" t="s">
         <v>389</v>
       </c>
@@ -5221,7 +5218,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="295" spans="1:3">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A295" s="4" t="s">
         <v>390</v>
       </c>
@@ -5232,7 +5229,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="296" spans="1:3">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A296" s="4" t="s">
         <v>391</v>
       </c>
@@ -5243,7 +5240,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="297" spans="1:3">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A297" s="4" t="s">
         <v>392</v>
       </c>
@@ -5254,7 +5251,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="298" spans="1:3">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A298" s="4" t="s">
         <v>393</v>
       </c>
@@ -5265,7 +5262,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="299" spans="1:3">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A299" s="4" t="s">
         <v>394</v>
       </c>
@@ -5276,7 +5273,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="300" spans="1:3">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A300" s="4" t="s">
         <v>395</v>
       </c>
@@ -5287,7 +5284,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="301" spans="1:3">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A301" s="4" t="s">
         <v>396</v>
       </c>
@@ -5298,7 +5295,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="302" spans="1:3">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A302" s="4" t="s">
         <v>397</v>
       </c>
@@ -5309,7 +5306,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="303" spans="1:3">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A303" s="4" t="s">
         <v>398</v>
       </c>
@@ -5320,7 +5317,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="304" spans="1:3">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A304" s="4" t="s">
         <v>399</v>
       </c>
@@ -5331,7 +5328,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="305" spans="1:3">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A305" s="4" t="s">
         <v>400</v>
       </c>
@@ -5342,7 +5339,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="306" spans="1:3">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A306" s="4" t="s">
         <v>401</v>
       </c>
@@ -5353,7 +5350,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="307" spans="1:3">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A307" s="4" t="s">
         <v>402</v>
       </c>
@@ -5364,7 +5361,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="308" spans="1:3">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A308" s="4" t="s">
         <v>403</v>
       </c>
@@ -5375,7 +5372,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="309" spans="1:3">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A309" s="4" t="s">
         <v>404</v>
       </c>
@@ -5386,7 +5383,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="310" spans="1:3">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A310" s="4" t="s">
         <v>405</v>
       </c>
@@ -5397,7 +5394,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="311" spans="1:3">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A311" s="4" t="s">
         <v>406</v>
       </c>
@@ -5408,7 +5405,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="312" spans="1:3">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A312" s="4" t="s">
         <v>407</v>
       </c>
@@ -5419,7 +5416,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="313" spans="1:3">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A313" s="4" t="s">
         <v>408</v>
       </c>
@@ -5430,7 +5427,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="314" spans="1:3">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A314" s="4" t="s">
         <v>409</v>
       </c>
@@ -5441,7 +5438,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="315" spans="1:3">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A315" s="4" t="s">
         <v>410</v>
       </c>
@@ -5452,7 +5449,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="316" spans="1:3">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A316" s="4" t="s">
         <v>411</v>
       </c>
@@ -5463,7 +5460,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="317" spans="1:3">
+    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A317" s="4" t="s">
         <v>412</v>
       </c>
@@ -5474,7 +5471,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="318" spans="1:3">
+    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A318" s="4" t="s">
         <v>413</v>
       </c>
@@ -5485,7 +5482,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="319" spans="1:3">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A319" s="4" t="s">
         <v>414</v>
       </c>
@@ -5496,7 +5493,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="320" spans="1:3">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A320" s="4" t="s">
         <v>415</v>
       </c>
@@ -5507,7 +5504,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="321" spans="1:3">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A321" s="4" t="s">
         <v>416</v>
       </c>
@@ -5518,7 +5515,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="322" spans="1:3">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A322" s="4" t="s">
         <v>417</v>
       </c>
@@ -5529,7 +5526,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="323" spans="1:3">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A323" s="4" t="s">
         <v>418</v>
       </c>
@@ -5540,7 +5537,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="324" spans="1:3">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A324" s="4" t="s">
         <v>419</v>
       </c>
@@ -5551,7 +5548,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="325" spans="1:3">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A325" s="4" t="s">
         <v>420</v>
       </c>
@@ -5562,7 +5559,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="326" spans="1:3">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A326" s="4" t="s">
         <v>421</v>
       </c>
@@ -5573,7 +5570,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="327" spans="1:3">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A327" s="4" t="s">
         <v>422</v>
       </c>
@@ -5584,7 +5581,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="328" spans="1:3">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A328" s="4" t="s">
         <v>423</v>
       </c>
@@ -5595,7 +5592,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="329" spans="1:3">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A329" s="4" t="s">
         <v>424</v>
       </c>
@@ -5606,7 +5603,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="330" spans="1:3">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A330" s="4" t="s">
         <v>425</v>
       </c>
@@ -5617,7 +5614,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="331" spans="1:3">
+    <row r="331" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A331" s="4" t="s">
         <v>426</v>
       </c>
@@ -5628,7 +5625,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="332" spans="1:3">
+    <row r="332" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A332" s="7" t="s">
         <v>121</v>
       </c>
@@ -5639,7 +5636,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="333" spans="1:3">
+    <row r="333" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A333" s="7" t="s">
         <v>122</v>
       </c>
@@ -5650,7 +5647,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="334" spans="1:3">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A334" s="7" t="s">
         <v>123</v>
       </c>
@@ -5661,7 +5658,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="335" spans="1:3">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A335" s="7" t="s">
         <v>124</v>
       </c>
@@ -5672,7 +5669,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="336" spans="1:3">
+    <row r="336" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A336" s="7" t="s">
         <v>125</v>
       </c>
@@ -5683,7 +5680,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="337" spans="1:3">
+    <row r="337" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A337" s="7" t="s">
         <v>126</v>
       </c>
@@ -5694,7 +5691,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="338" spans="1:3">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A338" s="7" t="s">
         <v>127</v>
       </c>
@@ -5705,7 +5702,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="339" spans="1:3">
+    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A339" s="8" t="s">
         <v>128</v>
       </c>
@@ -5716,7 +5713,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="340" spans="1:3">
+    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A340" s="8" t="s">
         <v>129</v>
       </c>
@@ -5727,7 +5724,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="341" spans="1:3">
+    <row r="341" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A341" s="8" t="s">
         <v>130</v>
       </c>
@@ -5738,7 +5735,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="342" spans="1:3">
+    <row r="342" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A342" s="8" t="s">
         <v>131</v>
       </c>
@@ -5749,7 +5746,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="343" spans="1:3">
+    <row r="343" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A343" s="8" t="s">
         <v>132</v>
       </c>
@@ -5760,7 +5757,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="344" spans="1:3">
+    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A344" s="8" t="s">
         <v>133</v>
       </c>
@@ -5771,7 +5768,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="345" spans="1:3">
+    <row r="345" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A345" s="8" t="s">
         <v>134</v>
       </c>
@@ -5782,7 +5779,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="346" spans="1:3">
+    <row r="346" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A346" s="8" t="s">
         <v>135</v>
       </c>
@@ -5793,7 +5790,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="347" spans="1:3">
+    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A347" s="8" t="s">
         <v>136</v>
       </c>
@@ -5804,7 +5801,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="348" spans="1:3">
+    <row r="348" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A348" s="8" t="s">
         <v>137</v>
       </c>
@@ -5815,7 +5812,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="349" spans="1:3">
+    <row r="349" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A349" s="8" t="s">
         <v>138</v>
       </c>
@@ -5826,7 +5823,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="350" spans="1:3">
+    <row r="350" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A350" s="8" t="s">
         <v>139</v>
       </c>
@@ -5837,7 +5834,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="351" spans="1:3">
+    <row r="351" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A351" s="8" t="s">
         <v>140</v>
       </c>
@@ -5848,7 +5845,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="352" spans="1:3">
+    <row r="352" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A352" s="8" t="s">
         <v>141</v>
       </c>
@@ -5859,7 +5856,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="353" spans="1:3">
+    <row r="353" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A353" s="8" t="s">
         <v>142</v>
       </c>
@@ -5870,7 +5867,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="354" spans="1:3">
+    <row r="354" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A354" s="8" t="s">
         <v>143</v>
       </c>
@@ -5881,7 +5878,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="355" spans="1:3">
+    <row r="355" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A355" s="8" t="s">
         <v>144</v>
       </c>
@@ -5892,7 +5889,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="356" spans="1:3">
+    <row r="356" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A356" s="8" t="s">
         <v>145</v>
       </c>
@@ -5903,7 +5900,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="357" spans="1:3">
+    <row r="357" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A357" s="8" t="s">
         <v>146</v>
       </c>
@@ -5914,7 +5911,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="358" spans="1:3">
+    <row r="358" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A358" s="8" t="s">
         <v>147</v>
       </c>
@@ -5925,7 +5922,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="359" spans="1:3">
+    <row r="359" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A359" s="8" t="s">
         <v>148</v>
       </c>
@@ -5936,7 +5933,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="360" spans="1:3">
+    <row r="360" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A360" s="8" t="s">
         <v>149</v>
       </c>
@@ -5947,7 +5944,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="361" spans="1:3">
+    <row r="361" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A361" s="8" t="s">
         <v>150</v>
       </c>
@@ -5958,7 +5955,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="362" spans="1:3">
+    <row r="362" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A362" s="8" t="s">
         <v>151</v>
       </c>
@@ -5969,7 +5966,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="363" spans="1:3">
+    <row r="363" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A363" s="8" t="s">
         <v>152</v>
       </c>
@@ -5980,7 +5977,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="364" spans="1:3">
+    <row r="364" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A364" s="8" t="s">
         <v>153</v>
       </c>
@@ -5991,7 +5988,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="365" spans="1:3">
+    <row r="365" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A365" s="8" t="s">
         <v>154</v>
       </c>
@@ -6002,7 +5999,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="366" spans="1:3">
+    <row r="366" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A366" s="8" t="s">
         <v>258</v>
       </c>
@@ -6013,7 +6010,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="367" spans="1:3">
+    <row r="367" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A367" s="8" t="s">
         <v>259</v>
       </c>
@@ -6024,7 +6021,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="368" spans="1:3">
+    <row r="368" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A368" s="8" t="s">
         <v>260</v>
       </c>
@@ -6035,7 +6032,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="369" spans="1:3">
+    <row r="369" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A369" s="8" t="s">
         <v>261</v>
       </c>
@@ -6046,7 +6043,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="370" spans="1:3">
+    <row r="370" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A370" s="8" t="s">
         <v>262</v>
       </c>
@@ -6057,7 +6054,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="371" spans="1:3">
+    <row r="371" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A371" s="8" t="s">
         <v>263</v>
       </c>
@@ -6068,7 +6065,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="372" spans="1:3">
+    <row r="372" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A372" s="8" t="s">
         <v>264</v>
       </c>
@@ -6079,7 +6076,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="373" spans="1:3">
+    <row r="373" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A373" s="8" t="s">
         <v>265</v>
       </c>
@@ -6090,7 +6087,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="374" spans="1:3">
+    <row r="374" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A374" s="8" t="s">
         <v>266</v>
       </c>
@@ -6101,7 +6098,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="375" spans="1:3">
+    <row r="375" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A375" s="8" t="s">
         <v>268</v>
       </c>
@@ -6112,7 +6109,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="376" spans="1:3">
+    <row r="376" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A376" s="8" t="s">
         <v>269</v>
       </c>
@@ -6123,7 +6120,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="377" spans="1:3">
+    <row r="377" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A377" s="8" t="s">
         <v>270</v>
       </c>
@@ -6134,7 +6131,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="378" spans="1:3">
+    <row r="378" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A378" s="8" t="s">
         <v>271</v>
       </c>
@@ -6145,7 +6142,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="379" spans="1:3">
+    <row r="379" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A379" s="8" t="s">
         <v>272</v>
       </c>
@@ -6156,7 +6153,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="380" spans="1:3">
+    <row r="380" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A380" s="8" t="s">
         <v>273</v>
       </c>
@@ -6167,7 +6164,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="381" spans="1:3">
+    <row r="381" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A381" s="8" t="s">
         <v>274</v>
       </c>
@@ -6178,7 +6175,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="382" spans="1:3">
+    <row r="382" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A382" s="8" t="s">
         <v>275</v>
       </c>
@@ -6189,7 +6186,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="383" spans="1:3">
+    <row r="383" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A383" s="8" t="s">
         <v>276</v>
       </c>
@@ -6200,7 +6197,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="384" spans="1:3">
+    <row r="384" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A384" s="8" t="s">
         <v>277</v>
       </c>
@@ -6211,7 +6208,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="385" spans="1:3">
+    <row r="385" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A385" s="8" t="s">
         <v>278</v>
       </c>
@@ -6222,7 +6219,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="386" spans="1:3">
+    <row r="386" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A386" s="8" t="s">
         <v>279</v>
       </c>
@@ -6233,7 +6230,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="387" spans="1:3">
+    <row r="387" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A387" s="8" t="s">
         <v>280</v>
       </c>
@@ -6244,7 +6241,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="388" spans="1:3">
+    <row r="388" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A388" s="8" t="s">
         <v>281</v>
       </c>
@@ -6255,7 +6252,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="389" spans="1:3">
+    <row r="389" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A389" s="8" t="s">
         <v>282</v>
       </c>
@@ -6266,7 +6263,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="390" spans="1:3">
+    <row r="390" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A390" s="8" t="s">
         <v>283</v>
       </c>
@@ -6277,7 +6274,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="391" spans="1:3">
+    <row r="391" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A391" s="8" t="s">
         <v>284</v>
       </c>
@@ -6288,7 +6285,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="392" spans="1:3">
+    <row r="392" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A392" s="8" t="s">
         <v>285</v>
       </c>
@@ -6299,7 +6296,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="393" spans="1:3">
+    <row r="393" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A393" s="8" t="s">
         <v>286</v>
       </c>
@@ -6310,7 +6307,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="394" spans="1:3">
+    <row r="394" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A394" s="8" t="s">
         <v>287</v>
       </c>
@@ -6321,7 +6318,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="395" spans="1:3">
+    <row r="395" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A395" s="8" t="s">
         <v>288</v>
       </c>
@@ -6332,7 +6329,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="396" spans="1:3">
+    <row r="396" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A396" s="8" t="s">
         <v>289</v>
       </c>
@@ -6343,7 +6340,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="397" spans="1:3">
+    <row r="397" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A397" s="8" t="s">
         <v>290</v>
       </c>
@@ -6354,7 +6351,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="398" spans="1:3">
+    <row r="398" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A398" s="8" t="s">
         <v>291</v>
       </c>
@@ -6365,7 +6362,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="399" spans="1:3">
+    <row r="399" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A399" s="8" t="s">
         <v>292</v>
       </c>
@@ -6376,7 +6373,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="400" spans="1:3">
+    <row r="400" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A400" s="8" t="s">
         <v>293</v>
       </c>
@@ -6387,7 +6384,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="401" spans="1:3">
+    <row r="401" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A401" s="8" t="s">
         <v>294</v>
       </c>
@@ -6398,7 +6395,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="402" spans="1:3">
+    <row r="402" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A402" s="8" t="s">
         <v>295</v>
       </c>
@@ -6409,7 +6406,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="403" spans="1:3">
+    <row r="403" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A403" s="8" t="s">
         <v>296</v>
       </c>
@@ -6420,7 +6417,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="404" spans="1:3">
+    <row r="404" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A404" s="8" t="s">
         <v>297</v>
       </c>
@@ -6431,7 +6428,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="405" spans="1:3">
+    <row r="405" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A405" s="8" t="s">
         <v>298</v>
       </c>
@@ -6442,7 +6439,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="406" spans="1:3">
+    <row r="406" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A406" s="8" t="s">
         <v>299</v>
       </c>
@@ -6453,7 +6450,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="407" spans="1:3">
+    <row r="407" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A407" s="8" t="s">
         <v>300</v>
       </c>
@@ -6464,7 +6461,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="408" spans="1:3">
+    <row r="408" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A408" s="8" t="s">
         <v>301</v>
       </c>
@@ -6475,7 +6472,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="409" spans="1:3">
+    <row r="409" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A409" s="8" t="s">
         <v>302</v>
       </c>
@@ -6486,7 +6483,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="410" spans="1:3">
+    <row r="410" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A410" s="8" t="s">
         <v>303</v>
       </c>
@@ -6497,7 +6494,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="411" spans="1:3">
+    <row r="411" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A411" s="8" t="s">
         <v>304</v>
       </c>
@@ -6508,7 +6505,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="412" spans="1:3">
+    <row r="412" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A412" s="8" t="s">
         <v>305</v>
       </c>
@@ -6519,7 +6516,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="413" spans="1:3">
+    <row r="413" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A413" s="8" t="s">
         <v>306</v>
       </c>
@@ -6530,7 +6527,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="414" spans="1:3">
+    <row r="414" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A414" s="8" t="s">
         <v>427</v>
       </c>
@@ -6541,7 +6538,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="415" spans="1:3">
+    <row r="415" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A415" s="8" t="s">
         <v>428</v>
       </c>
@@ -6552,7 +6549,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="416" spans="1:3">
+    <row r="416" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A416" s="8" t="s">
         <v>429</v>
       </c>
@@ -6563,7 +6560,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="417" spans="1:3">
+    <row r="417" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A417" s="8" t="s">
         <v>430</v>
       </c>
@@ -6574,7 +6571,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="418" spans="1:3">
+    <row r="418" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A418" s="8" t="s">
         <v>431</v>
       </c>
@@ -6585,7 +6582,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="419" spans="1:3">
+    <row r="419" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A419" s="8" t="s">
         <v>432</v>
       </c>
@@ -6596,7 +6593,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="420" spans="1:3">
+    <row r="420" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A420" s="8" t="s">
         <v>433</v>
       </c>
@@ -6607,7 +6604,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="421" spans="1:3">
+    <row r="421" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A421" s="8" t="s">
         <v>434</v>
       </c>
@@ -6618,7 +6615,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="422" spans="1:3">
+    <row r="422" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A422" s="8" t="s">
         <v>435</v>
       </c>
@@ -6629,7 +6626,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="423" spans="1:3">
+    <row r="423" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A423" s="8" t="s">
         <v>436</v>
       </c>
@@ -6640,7 +6637,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="424" spans="1:3">
+    <row r="424" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A424" s="8" t="s">
         <v>437</v>
       </c>
@@ -6651,7 +6648,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="425" spans="1:3">
+    <row r="425" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A425" s="4" t="s">
         <v>438</v>
       </c>
@@ -6662,7 +6659,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="426" spans="1:3">
+    <row r="426" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A426" s="8" t="s">
         <v>439</v>
       </c>
@@ -6673,7 +6670,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="427" spans="1:3">
+    <row r="427" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A427" s="8" t="s">
         <v>440</v>
       </c>
@@ -6684,7 +6681,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="428" spans="1:3">
+    <row r="428" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A428" s="8" t="s">
         <v>441</v>
       </c>
@@ -6695,7 +6692,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="429" spans="1:3">
+    <row r="429" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A429" s="8" t="s">
         <v>442</v>
       </c>
@@ -6706,7 +6703,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="430" spans="1:3">
+    <row r="430" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A430" s="8" t="s">
         <v>443</v>
       </c>
@@ -6717,7 +6714,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="431" spans="1:3">
+    <row r="431" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A431" s="8" t="s">
         <v>444</v>
       </c>
@@ -6728,7 +6725,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="432" spans="1:3">
+    <row r="432" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A432" s="8" t="s">
         <v>445</v>
       </c>
@@ -6739,7 +6736,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="433" spans="1:3">
+    <row r="433" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A433" s="8" t="s">
         <v>446</v>
       </c>
@@ -6750,7 +6747,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="434" spans="1:3">
+    <row r="434" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A434" s="8" t="s">
         <v>447</v>
       </c>
@@ -6761,7 +6758,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="435" spans="1:3">
+    <row r="435" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A435" s="8" t="s">
         <v>448</v>
       </c>
@@ -6772,7 +6769,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="436" spans="1:3">
+    <row r="436" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A436" s="8" t="s">
         <v>449</v>
       </c>
@@ -6783,7 +6780,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="437" spans="1:3">
+    <row r="437" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A437" s="8" t="s">
         <v>450</v>
       </c>
@@ -6794,7 +6791,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="438" spans="1:3">
+    <row r="438" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A438" s="8" t="s">
         <v>451</v>
       </c>
@@ -6805,7 +6802,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="439" spans="1:3">
+    <row r="439" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A439" s="8" t="s">
         <v>452</v>
       </c>
@@ -6816,7 +6813,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="440" spans="1:3">
+    <row r="440" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A440" s="8" t="s">
         <v>453</v>
       </c>
@@ -6827,7 +6824,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="441" spans="1:3">
+    <row r="441" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A441" s="8" t="s">
         <v>454</v>
       </c>
@@ -6838,7 +6835,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="442" spans="1:3">
+    <row r="442" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A442" s="8" t="s">
         <v>455</v>
       </c>
@@ -6849,7 +6846,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="443" spans="1:3">
+    <row r="443" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A443" s="8" t="s">
         <v>456</v>
       </c>
@@ -6860,7 +6857,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="444" spans="1:3">
+    <row r="444" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A444" s="8" t="s">
         <v>457</v>
       </c>
@@ -6871,7 +6868,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="445" spans="1:3">
+    <row r="445" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A445" s="8" t="s">
         <v>458</v>
       </c>
@@ -6882,7 +6879,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="446" spans="1:3">
+    <row r="446" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A446" s="8" t="s">
         <v>459</v>
       </c>
@@ -6893,7 +6890,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="447" spans="1:3">
+    <row r="447" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A447" s="8" t="s">
         <v>460</v>
       </c>
@@ -6904,7 +6901,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="448" spans="1:3">
+    <row r="448" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A448" s="8" t="s">
         <v>464</v>
       </c>
@@ -6915,7 +6912,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="449" spans="1:3">
+    <row r="449" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A449" s="8" t="s">
         <v>466</v>
       </c>
@@ -6926,7 +6923,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="450" spans="1:3">
+    <row r="450" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A450" s="8" t="s">
         <v>468</v>
       </c>
@@ -6937,7 +6934,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="451" spans="1:3">
+    <row r="451" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A451" s="8" t="s">
         <v>470</v>
       </c>
@@ -6948,7 +6945,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="452" spans="1:3">
+    <row r="452" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A452" s="9" t="s">
         <v>155</v>
       </c>
@@ -6959,7 +6956,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="453" spans="1:3">
+    <row r="453" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A453" s="9" t="s">
         <v>156</v>
       </c>
@@ -6970,7 +6967,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="454" spans="1:3">
+    <row r="454" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A454" s="9" t="s">
         <v>307</v>
       </c>
@@ -6981,7 +6978,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="455" spans="1:3">
+    <row r="455" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A455" s="9" t="s">
         <v>308</v>
       </c>
@@ -6992,7 +6989,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="456" spans="1:3">
+    <row r="456" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A456" s="9" t="s">
         <v>309</v>
       </c>
@@ -7003,7 +7000,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="457" spans="1:3">
+    <row r="457" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A457" s="9" t="s">
         <v>310</v>
       </c>
@@ -7014,7 +7011,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="458" spans="1:3">
+    <row r="458" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A458" s="9" t="s">
         <v>311</v>
       </c>
@@ -7025,7 +7022,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="459" spans="1:3">
+    <row r="459" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A459" s="9" t="s">
         <v>461</v>
       </c>
@@ -7036,7 +7033,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="460" spans="1:3">
+    <row r="460" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A460" s="8" t="s">
         <v>462</v>
       </c>
@@ -7047,7 +7044,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="461" spans="1:3">
+    <row r="461" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A461" s="9" t="s">
         <v>463</v>
       </c>
@@ -7058,7 +7055,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="462" spans="1:3">
+    <row r="462" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A462" s="8" t="s">
         <v>465</v>
       </c>
@@ -7069,7 +7066,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="463" spans="1:3">
+    <row r="463" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A463" s="9" t="s">
         <v>467</v>
       </c>
@@ -7080,7 +7077,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="464" spans="1:3">
+    <row r="464" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A464" s="9" t="s">
         <v>469</v>
       </c>

</xml_diff>